<commit_message>
Regenerated audit pack with evidence columns
</commit_message>
<xml_diff>
--- a/review/audit_pack.xlsx
+++ b/review/audit_pack.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rejects" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Accepts'!$A$2:$J$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rejects'!$A$2:$J$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Accepts'!$A$2:$M$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rejects'!$A$2:$M$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,19 +481,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,25 +534,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>OSCR purposes</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Objects / Activities</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Form / UKCAT</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>Model verdict</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Model reason</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -575,21 +593,32 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of citizenship or community development'"]</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['SL']</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Windfarm legacy SCIO likely distributes community benefit funds as grants</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="4" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr"/>
+      <c r="M3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -611,21 +640,32 @@
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education'"]</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['RL201', 'ED']</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="J4" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Guildry likely distributes funds to local causes</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -647,21 +687,32 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of religion','the advancement of citizenship or community development','the advancement of human rights, conflict resolution or reconciliation','the advancement of environmental protection or improvement','any other purpose that may reasonably be regarded as analogous to any of the preceding purposes'"]</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'RL300', 'SL', 'RL301', 'EN', 'BE']</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Trust with broad charitable purposes likely makes grants</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="4" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="3" t="n">
@@ -683,21 +734,32 @@
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>['The advancement of education', 'The advancement of the arts', 'culture', 'heritage or science', 'The advancement of environmental protection or improvement']</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Trust Deed or Declaration of Trust / ['ED', 'AR', 'EN']</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="J6" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Trust with broad purposes likely makes grants</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -719,21 +781,32 @@
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of citizenship or community development'"]</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'SL']</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Trust with poverty relief and community development purposes likely grants.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="3" t="n">
@@ -755,21 +828,32 @@
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="J8" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Trust with education/arts purposes typically makes grants</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="L8" s="3" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -791,21 +875,32 @@
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of citizenship or community development'"]</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['ED', 'SL']</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="J9" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Foundation makes grants to advance education and community development.</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="3" t="n">
@@ -827,21 +922,32 @@
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of education'"]</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['ED']</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="J10" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Trust with education purpose likely provides grants</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -863,21 +969,32 @@
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>['The prevention or relief of poverty', 'The advancement of education', 'The advancement of health or the saving of lives', 'The relief of those in need by reason of youth', 'age', 'ill-health', 'disability', 'financial hardship or other disadvantage']</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Memorandum and Articles / ['ED', 'HE', 'RL201', 'SL']</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="J11" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Foundation with broad charitable purposes likely grants to other organisations.</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="4" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="3" t="n">
@@ -899,21 +1016,32 @@
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of citizenship or community development','the advancement of public participation in sport','the advancement of environmental protection or improvement','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'ED', 'SL', 'CA300', 'EN', 'HE']</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="J12" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Rotary club trust fund likely distributes grants to community causes.</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -935,21 +1063,32 @@
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of health','the advancement of citizenship or community development','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['HE', 'SL', 'RL201']</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="J13" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Trust likely provides grants to organisations based on name and purposes</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr"/>
+      <c r="M13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="3" t="n">
@@ -971,21 +1110,32 @@
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of environmental protection or improvement'"]</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['EN']</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="J14" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>Trust likely funds environmental projects via grants.</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr"/>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -1007,21 +1157,32 @@
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['RL201', 'ED', 'HE']</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="J15" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>International aid agency funding partner organisations overseas</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="3" t="n">
@@ -1043,21 +1204,32 @@
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of public participation in sport'"]</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['CA300']</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="J16" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Sports council likely distributes grants to local sports clubs.</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -1079,21 +1251,32 @@
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of citizenship or community development','the advancement of public participation in sport','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended'"]</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['RL201', 'ED', 'SL', 'CA300']</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G17" s="3" t="n">
+      <c r="J17" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Foundation likely provides grants for rugby and community projects.</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="3" t="n">
@@ -1115,21 +1298,32 @@
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="J18" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Trust funds education and science, likely grants to researchers/organisations.</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr"/>
+      <c r="M18" s="4" t="inlineStr"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -1151,21 +1345,32 @@
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G19" s="3" t="n">
+      <c r="J19" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Trust likely funds mathematical journal and research grants.</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="4" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr"/>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="3" t="n">
@@ -1187,21 +1392,32 @@
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of health','the saving of lives','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage','the advancement of animal welfare'"]</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['HE', 'HE201', 'RL201', 'AN']</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n">
+      <c r="J20" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Charitable trust with broad purposes, likely grantmaking</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr"/>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -1223,21 +1439,32 @@
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of the arts, heritage, culture or science','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['RL201', 'ED', 'CA', 'HE']</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G21" s="3" t="n">
+      <c r="J21" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Rotary club trust funds typically make grants to other organisations.</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="4" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr"/>
+      <c r="M21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="3" t="n">
@@ -1259,21 +1486,32 @@
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of health'"]</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['HE']</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n">
+      <c r="J22" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="K22" s="4" t="inlineStr">
         <is>
           <t>Foundation likely funds cancer research grants</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr"/>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="3" t="n">
@@ -1295,21 +1533,32 @@
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of religion','the saving of lives','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['RL201', 'ED', 'RL300', 'HE201', 'HE']</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="J23" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Trust with broad charitable purposes likely provides grants</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="4" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr"/>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="3" t="n">
@@ -1331,21 +1580,32 @@
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of health','the advancement of citizenship or community development','the advancement of the arts, heritage, culture or science','the advancement of public participation in sport','the advancement of environmental protection or improvement','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['RL201', 'ED', 'HE', 'SL', 'CA', 'CA300', 'EN']</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G24" s="3" t="n">
+      <c r="J24" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>Foundation with broad charitable purposes, likely grants to community groups</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr"/>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -1367,21 +1627,32 @@
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['ED', 'RL201', 'HE']</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="J25" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Trust likely provides grants to children's causes</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="4" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr"/>
+      <c r="M25" s="4" t="inlineStr"/>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="3" t="n">
@@ -1403,21 +1674,32 @@
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="J26" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>Trust likely funds historical research and publications through grants.</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr"/>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -1439,21 +1721,32 @@
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of health','the advancement of citizenship or community development','the advancement of the arts, heritage, culture or science','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage','any other purpose that may reasonably be regarded as analogous to any of the preceding purposes'"]</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'ED', 'HE', 'SL', 'CA', 'BE']</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G27" s="3" t="n">
+      <c r="J27" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Rotary club charitable trust likely makes grants to community causes.</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="4" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr"/>
+      <c r="M27" s="4" t="inlineStr"/>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="3" t="n">
@@ -1475,21 +1768,32 @@
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>['The prevention or relief of poverty', 'The advancement of education', 'The advancement of religion']</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Trust Deed or Declaration of Trust / ['ED', 'RL300', 'RL201']</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="J28" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>Charitable trust with broad purposes likely makes grants.</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="4" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr"/>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="3" t="n">
@@ -1511,21 +1815,32 @@
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>["'the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['CA']</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G29" s="3" t="n">
+      <c r="J29" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="K29" s="4" t="inlineStr">
         <is>
           <t>Foundation likely supports arts via grants to makers.</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr"/>
+      <c r="M29" s="4" t="inlineStr"/>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="3" t="n">
@@ -1547,21 +1862,32 @@
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of health','the advancement of citizenship or community development','the promotion of equality and diversity'"]</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'ED', 'HE', 'SL', 'RL301']</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="J30" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="K30" s="4" t="inlineStr">
         <is>
           <t>Foundation with broad charitable purposes, likely grantmaking.</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="4" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr"/>
+      <c r="M30" s="4" t="inlineStr"/>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -1583,21 +1909,32 @@
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of citizenship or community development','the advancement of the arts, heritage, culture or science','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended','the advancement of environmental protection or improvement','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['RL201', 'ED', 'SL', 'CA', 'CA300', 'EN', 'HE']</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n">
+      <c r="J31" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="K31" s="4" t="inlineStr">
         <is>
           <t>Community trust likely distributes grants from wind farm revenues.</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr"/>
+      <c r="M31" s="4" t="inlineStr"/>
     </row>
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="3" t="n">
@@ -1619,28 +1956,39 @@
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of religion','the advancement of health','the advancement of citizenship or community development','the advancement of the arts, heritage, culture or science','the advancement of public participation in sport','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended','the promotion of equality and diversity','the advancement of environmental protection or improvement','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'ED', 'RL300', 'HE', 'SL', 'CA', 'CA300', 'RL301', 'EN']</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>GRANTMAKER</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="J32" s="3" t="n">
         <v>0.95</v>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="K32" s="4" t="inlineStr">
         <is>
           <t>Charitable trust with broad purposes, typically distributes grants</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="4" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J32"/>
+  <autoFilter ref="A2:M32"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G3:G32">
+  <conditionalFormatting sqref="J3:J32">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.85</formula>
     </cfRule>
@@ -1656,19 +2004,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1706,25 +2057,40 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>OSCR purposes</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Objects / Activities</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Form / UKCAT</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>Model verdict</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Model reason</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Human</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1750,21 +2116,32 @@
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of religion'"]</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['RL201', 'ED', 'RL300']</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="J3" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity in Uganda, not grantmaking to other organisations.</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="6" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr"/>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="5" t="n">
@@ -1786,21 +2163,32 @@
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="J4" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Educational charity providing philosophy courses, not grantmaking to other organisations.</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="6" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="5" t="n">
@@ -1822,21 +2210,32 @@
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of religion'"]</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL300']</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>Church advancing religion, not giving grants to organisations</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="6" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="5" t="n">
@@ -1858,21 +2257,32 @@
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of the arts, heritage, culture or science','any other purpose that may reasonably be regarded as analogous to any of the preceding purposes'"]</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['CA', 'BE']</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="J6" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Male voice choir, not a grantmaking organisation</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="5" t="n">
@@ -1894,21 +2304,32 @@
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of health','the advancement of citizenship or community development','the advancement of public participation in sport','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended'"]</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['ED', 'HE', 'SL', 'CA300']</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="J7" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity advancing sport, education, health, community development directly.</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="5" t="n">
@@ -1930,21 +2351,32 @@
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of citizenship or community development','the advancement of the arts, heritage, culture or science','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended','the advancement of environmental protection or improvement','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['SL', 'CA', 'CA300', 'EN', 'RL201', 'HE']</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="J8" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>Community development charity delivering services, not primarily grantmaking</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="5" t="n">
@@ -1966,21 +2398,32 @@
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the promotion of religious or racial harmony'"]</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['ED', 'RL300', 'RL301']</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="J9" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Educational/religious charity likely delivers own programs, not grants.</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr"/>
+      <c r="M9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -2002,21 +2445,32 @@
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of citizenship or community development','the advancement of environmental protection or improvement'"]</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['SL', 'EN']</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="J10" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>Civic trust likely runs projects, not primarily grants to organisations.</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="6" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="45" customHeight="1">
       <c r="A11" s="5" t="n">
@@ -2038,21 +2492,32 @@
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of health','the advancement of human rights, conflict resolution or reconciliation','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['ED', 'HE', 'RL301', 'RL201']</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="J11" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Likely an umbrella/advocacy charity, not primarily a grantmaker</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="6" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr"/>
+      <c r="M11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="5" t="n">
@@ -2074,21 +2539,32 @@
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of citizenship or community development','the advancement of public participation in sport','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended'"]</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'ED', 'SL', 'CA300']</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="J12" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Likely council-run educational trust, not grantmaking to other organisations.</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr"/>
+      <c r="M12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="5" t="n">
@@ -2110,21 +2586,32 @@
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of religion','the promotion of religious or racial harmony'"]</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['RL300', 'RL301']</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="J13" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Church advancing religion, not giving grants to organizations</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="6" t="inlineStr"/>
+      <c r="L13" s="5" t="inlineStr"/>
+      <c r="M13" s="6" t="inlineStr"/>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="5" t="n">
@@ -2146,21 +2633,32 @@
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of health','the promotion of equality and diversity','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['HE', 'RL301', 'RL201']</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="J14" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity for disabled people, not a grantmaker.</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="6" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="5" t="n">
@@ -2182,21 +2680,32 @@
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['RL201', 'CA300', 'HE']</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="J15" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity focused on poverty relief and recreational activities.</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="6" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr"/>
+      <c r="M15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="45" customHeight="1">
       <c r="A16" s="5" t="n">
@@ -2218,21 +2727,32 @@
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="J16" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Provides music education and performance opportunities, not grants to other organisations.</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr"/>
-      <c r="J16" s="6" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
+      <c r="M16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="5" t="n">
@@ -2254,21 +2774,32 @@
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of education','the advancement of health','the advancement of human rights, conflict resolution or reconciliation'"]</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['RL201', 'ED', 'HE', 'RL301']</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="J17" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>UNICEF UK delivers programmes and advocacy, not primarily grants to other organisations.</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="6" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="5" t="n">
@@ -2290,21 +2821,32 @@
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of health'"]</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['HE']</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="J18" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>Likely service-delivery cancer charity, not grantmaker</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="6" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
+      <c r="M18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="45" customHeight="1">
       <c r="A19" s="5" t="n">
@@ -2326,21 +2868,32 @@
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of religion'"]</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['ED', 'RL300']</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="J19" s="5" t="n">
         <v>0.7</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Education and religion purposes suggest service-delivery, not grantmaking</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr"/>
     </row>
     <row r="20" ht="45" customHeight="1">
       <c r="A20" s="5" t="n">
@@ -2362,21 +2915,32 @@
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="J20" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Promotes Gaelic language and culture, likely service delivery not grantmaking.</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="6" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr"/>
     </row>
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="5" t="n">
@@ -2398,21 +2962,32 @@
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr"/>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of health','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['HE', 'RL201']</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="J21" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity supporting kidney patients, not primarily a grantmaker</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr"/>
+      <c r="M21" s="6" t="inlineStr"/>
     </row>
     <row r="22" ht="45" customHeight="1">
       <c r="A22" s="5" t="n">
@@ -2434,21 +3009,32 @@
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr"/>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>['The advancement of health or the saving of lives', 'The relief of those in need by reason of youth', 'age', 'ill-health', 'disability', 'financial hardship or other disadvantage']</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Memorandum and Articles / ['HE', 'RL201', 'SL']</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="J22" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity providing oxygen therapy directly to beneficiaries.</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="6" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr"/>
+      <c r="M22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="45" customHeight="1">
       <c r="A23" s="5" t="n">
@@ -2470,21 +3056,32 @@
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr"/>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of health','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['HE', 'RL201']</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G23" s="5" t="n">
+      <c r="J23" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity supporting children's hospital, not grantmaking to other organizations.</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="6" t="inlineStr"/>
+      <c r="L23" s="5" t="inlineStr"/>
+      <c r="M23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="45" customHeight="1">
       <c r="A24" s="5" t="n">
@@ -2506,21 +3103,32 @@
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr"/>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of citizenship or community development','the advancement of the arts, heritage, culture or science','the provision of recreational facilities, or the organisation of recreational activities, with the object of improving the conditions of life for the persons for whom the facilities or activities are primarily intended','the advancement of environmental protection or improvement'"]</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['SL', 'CA', 'CA300', 'EN']</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="J24" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>Community association providing facilities and activities, not grants</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr"/>
-      <c r="J24" s="6" t="inlineStr"/>
+      <c r="L24" s="5" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr"/>
     </row>
     <row r="25" ht="45" customHeight="1">
       <c r="A25" s="5" t="n">
@@ -2542,21 +3150,32 @@
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr"/>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of the arts, heritage, culture or science'"]</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['ED', 'CA']</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G25" s="5" t="n">
+      <c r="J25" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>Choral society, performs music; not a grantmaker</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="6" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr"/>
     </row>
     <row r="26" ht="45" customHeight="1">
       <c r="A26" s="5" t="n">
@@ -2578,21 +3197,32 @@
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr"/>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>['The advancement of education', 'The advancement of the arts', 'culture', 'heritage or science']</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>['ED', 'AR']</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="J26" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Likely cultural/educational charity, not grantmaker</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr"/>
-      <c r="J26" s="6" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr"/>
     </row>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="5" t="n">
@@ -2614,21 +3244,32 @@
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr"/>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of health'"]</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Company (the charity is registered with Companies House) / ['ED', 'HE']</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G27" s="5" t="n">
+      <c r="J27" s="5" t="n">
         <v>0.8</v>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>Professional membership association, not primarily a grantmaker</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="6" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr"/>
+      <c r="M27" s="6" t="inlineStr"/>
     </row>
     <row r="28" ht="45" customHeight="1">
       <c r="A28" s="5" t="n">
@@ -2650,21 +3291,32 @@
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr"/>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the saving of lives','the relief of those in need by reason of age, ill-health, disability, financial hardship or other disadvantage'"]</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>SCIO (Scottish Charitable Incorporated Organisation) / ['RL201', 'HE201', 'HE']</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G28" s="5" t="n">
+      <c r="J28" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>Service-delivery charity focused on poverty relief and saving lives.</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="6" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr"/>
+      <c r="M28" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="45" customHeight="1">
       <c r="A29" s="5" t="n">
@@ -2686,21 +3338,32 @@
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr"/>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>['The advancement of health or the saving of lives', 'The relief of those in need by reason of youth', 'age', 'ill-health', 'disability', 'financial hardship or other disadvantage']</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Memorandum and Articles / ['HE', 'RL201', 'SL']</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G29" s="5" t="n">
+      <c r="J29" s="5" t="n">
         <v>0.6</v>
       </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>Purposes suggest direct service delivery, not grantmaking.</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="6" t="inlineStr"/>
+      <c r="L29" s="5" t="inlineStr"/>
+      <c r="M29" s="6" t="inlineStr"/>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="5" t="n">
@@ -2722,21 +3385,32 @@
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr"/>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>["'the prevention or relief of poverty','the advancement of religion'"]</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Trust (founding document is a deed of trust) (other than educational endowment) / ['RL201', 'RL300']</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="J30" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>Church advancing religion, not primarily giving grants to organizations</t>
         </is>
       </c>
-      <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="6" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr"/>
+      <c r="M30" s="6" t="inlineStr"/>
     </row>
     <row r="31" ht="45" customHeight="1">
       <c r="A31" s="5" t="n">
@@ -2758,21 +3432,32 @@
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr"/>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of religion'"]</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['RL300']</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G31" s="5" t="n">
+      <c r="J31" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>Baptist church advancing religion, not giving grants to organizations</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="6" t="inlineStr"/>
+      <c r="L31" s="5" t="inlineStr"/>
+      <c r="M31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="45" customHeight="1">
       <c r="A32" s="5" t="n">
@@ -2794,28 +3479,39 @@
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr"/>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>["'the advancement of education','the advancement of health','the advancement of public participation in sport'"]</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Unincorporated association / ['ED', 'HE', 'CA300']</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>NOT grantmaker</t>
         </is>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="J32" s="5" t="n">
         <v>0.95</v>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="K32" s="6" t="inlineStr">
         <is>
           <t>PTA fundraising for its own school, not granting to others</t>
         </is>
       </c>
-      <c r="I32" s="5" t="inlineStr"/>
-      <c r="J32" s="6" t="inlineStr"/>
+      <c r="L32" s="5" t="inlineStr"/>
+      <c r="M32" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J32"/>
+  <autoFilter ref="A2:M32"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G3:G32">
+  <conditionalFormatting sqref="J3:J32">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0.85</formula>
     </cfRule>

</xml_diff>